<commit_message>
fix: backtest partition label uses majority flag (not any-match)
Previous logic: if ANY oot sample → label as OOT (wrong for mixed months)
New logic: use dominant (most frequent) flag in the month

94 tests pass.
</commit_message>
<xml_diff>
--- a/report_100k.xlsx
+++ b/report_100k.xlsx
@@ -5481,7 +5481,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -5554,7 +5554,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -5700,7 +5700,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -5773,7 +5773,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -5846,7 +5846,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -5919,7 +5919,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -5992,7 +5992,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -6065,7 +6065,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -6138,7 +6138,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -6211,7 +6211,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -6284,7 +6284,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">

</xml_diff>

<commit_message>
refactor: Sheet 1 merge train+test into single 训练测试集 row per month
- Use majority flag per month to determine label
- train and test merged into one row (训练测试集)
- Months don't share train/test and oot/oos in real data
</commit_message>
<xml_diff>
--- a/report_100k.xlsx
+++ b/report_100k.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>训练集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -518,407 +518,359 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>5001</v>
+        <v>6232</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>5099</v>
+        <v>6358</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>1.92%</t>
+          <t>1.98%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>测试集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>202501</t>
+          <t>202502</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1231</v>
+        <v>6155</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>28</v>
+        <v>115</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1259</v>
+        <v>6270</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>1.83%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>202501</t>
+          <t>202503</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1642</v>
+        <v>6113</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>37</v>
+        <v>125</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1679</v>
+        <v>6238</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>2.00%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>压测</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>202501</t>
+          <t>202504</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>405</v>
+        <v>6195</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>6</v>
+        <v>115</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>411</v>
+        <v>6310</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1.46%</t>
+          <t>1.82%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>训练集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>202502</t>
+          <t>202505</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>4938</v>
+        <v>6184</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>5030</v>
+        <v>6303</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>1.83%</t>
+          <t>1.89%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>测试集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>202502</t>
+          <t>202506</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1217</v>
+        <v>6066</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1240</v>
+        <v>6182</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>1.85%</t>
+          <t>1.88%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>202502</t>
+          <t>202507</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1630</v>
+        <v>6023</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>29</v>
+        <v>118</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1659</v>
+        <v>6141</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>1.92%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>压测</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>202502</t>
+          <t>202508</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>405</v>
+        <v>6174</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>8</v>
+        <v>135</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>413</v>
+        <v>6309</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>1.94%</t>
+          <t>2.14%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>训练集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>202503</t>
+          <t>202509</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>4892</v>
+        <v>6121</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>4994</v>
+        <v>6250</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>2.06%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>测试集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>202503</t>
+          <t>202510</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1221</v>
+        <v>6054</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>1244</v>
+        <v>6172</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>1.85%</t>
+          <t>1.91%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>跨时间验证集</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>202503</t>
+          <t>202511</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1646</v>
+        <v>6169</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>24</v>
+        <v>121</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1670</v>
+        <v>6290</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.92%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>压测</t>
+          <t>训练测试集</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>202503</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>399</v>
+        <v>6149</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>6</v>
+        <v>138</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>405</v>
+        <v>6287</v>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>2.20%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>202504</t>
-        </is>
-      </c>
+          <t>总计</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="3" t="n">
-        <v>4954</v>
+        <v>98055</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>91</v>
+        <v>1945</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>5045</v>
+        <v>100000</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>1.80%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>202504</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>1241</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>1265</v>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>1.90%</t>
+          <t>1.94%</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>202504</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>1675</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>1704</v>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>1.70%</t>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>modeling_score</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>202504</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>430</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>433</v>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>0.69%</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>样本数据集划分标签</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>好</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>坏</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>总数</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>坏占比</t>
         </is>
       </c>
     </row>
@@ -928,21 +880,16 @@
           <t>训练集</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>202505</t>
-        </is>
+      <c r="B19" s="3" t="n">
+        <v>58836</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>4966</v>
+        <v>1168</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>99</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>5065</v>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
+        <v>60004</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>1.95%</t>
         </is>
@@ -954,23 +901,18 @@
           <t>测试集</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>202505</t>
-        </is>
+      <c r="B20" s="3" t="n">
+        <v>14799</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1218</v>
+        <v>307</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>1238</v>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>1.62%</t>
+        <v>15106</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>2.03%</t>
         </is>
       </c>
     </row>
@@ -980,915 +922,37 @@
           <t>跨时间验证集</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>202505</t>
-        </is>
+      <c r="B21" s="3" t="n">
+        <v>19547</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1597</v>
+        <v>379</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>1623</v>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>1.60%</t>
+        <v>19926</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>1.90%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>202505</t>
-        </is>
+          <t>总计</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>98055</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>407</v>
+        <v>1945</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>419</v>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>2.86%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>202506</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>4844</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>89</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>4933</v>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>1.80%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>202506</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>1222</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>1249</v>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>2.16%</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>202506</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>1615</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>1643</v>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>1.70%</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>202506</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>367</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>373</v>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>1.61%</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>202507</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>4818</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>93</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>4911</v>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>1.89%</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>202507</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>1205</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>1230</v>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>2.03%</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>202507</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>1593</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>1636</v>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>2.63%</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>202507</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>410</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>415</v>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>1.20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>202508</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>4905</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>102</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>5007</v>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>2.04%</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>202508</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>1269</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>33</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>1302</v>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>2.53%</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>202508</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>1650</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>1693</v>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>2.54%</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>202508</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="n">
-        <v>418</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>430</v>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>2.79%</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>202509</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="n">
-        <v>4907</v>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>96</v>
-      </c>
-      <c r="E35" s="3" t="n">
-        <v>5003</v>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>1.92%</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>202509</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="n">
-        <v>1214</v>
-      </c>
-      <c r="D36" s="3" t="n">
-        <v>33</v>
-      </c>
-      <c r="E36" s="3" t="n">
-        <v>1247</v>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>2.65%</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>202509</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="n">
-        <v>1641</v>
-      </c>
-      <c r="D37" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>1671</v>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>1.80%</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>202509</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="n">
-        <v>426</v>
-      </c>
-      <c r="D38" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>435</v>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>2.07%</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>202510</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n">
-        <v>4825</v>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>97</v>
-      </c>
-      <c r="E39" s="3" t="n">
-        <v>4922</v>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>1.97%</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>202510</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>1229</v>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>1250</v>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>1.68%</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>202510</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="n">
-        <v>1671</v>
-      </c>
-      <c r="D41" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="E41" s="3" t="n">
-        <v>1705</v>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>1.99%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>202510</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>399</v>
-      </c>
-      <c r="D42" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="E42" s="3" t="n">
-        <v>406</v>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>1.72%</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>202511</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n">
-        <v>4910</v>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="E43" s="3" t="n">
-        <v>5010</v>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>2.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>202511</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="n">
-        <v>1259</v>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="E44" s="3" t="n">
-        <v>1280</v>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>1.64%</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>202511</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="n">
-        <v>1561</v>
-      </c>
-      <c r="D45" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="E45" s="3" t="n">
-        <v>1586</v>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>1.58%</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>202511</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="n">
-        <v>429</v>
-      </c>
-      <c r="D46" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E46" s="3" t="n">
-        <v>437</v>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>1.83%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>202512</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="n">
-        <v>4876</v>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>109</v>
-      </c>
-      <c r="E47" s="3" t="n">
-        <v>4985</v>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>2.19%</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>202512</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="n">
-        <v>1273</v>
-      </c>
-      <c r="D48" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="E48" s="3" t="n">
-        <v>1302</v>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>2.23%</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>202512</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="n">
-        <v>1626</v>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="E49" s="3" t="n">
-        <v>1657</v>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>1.87%</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>压测</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>202512</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="n">
-        <v>378</v>
-      </c>
-      <c r="D50" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="E50" s="3" t="n">
-        <v>387</v>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>2.33%</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>总计</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr"/>
-      <c r="C51" s="3" t="n">
-        <v>98055</v>
-      </c>
-      <c r="D51" s="3" t="n">
-        <v>1945</v>
-      </c>
-      <c r="E51" s="3" t="n">
         <v>100000</v>
       </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>1.94%</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="inlineStr">
-        <is>
-          <t>modeling_score</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>样本数据集划分标签</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>好</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>坏</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>总数</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>坏占比</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>训练集</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n">
-        <v>58836</v>
-      </c>
-      <c r="C55" s="3" t="n">
-        <v>1168</v>
-      </c>
-      <c r="D55" s="3" t="n">
-        <v>60004</v>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>1.95%</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>测试集</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="n">
-        <v>14799</v>
-      </c>
-      <c r="C56" s="3" t="n">
-        <v>307</v>
-      </c>
-      <c r="D56" s="3" t="n">
-        <v>15106</v>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>2.03%</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>跨时间验证集</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="n">
-        <v>19547</v>
-      </c>
-      <c r="C57" s="3" t="n">
-        <v>379</v>
-      </c>
-      <c r="D57" s="3" t="n">
-        <v>19926</v>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>1.90%</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>总计</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="n">
-        <v>98055</v>
-      </c>
-      <c r="C58" s="3" t="n">
-        <v>1945</v>
-      </c>
-      <c r="D58" s="3" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>1.94%</t>
         </is>

</xml_diff>

<commit_message>
refactor: Sheet 1 section names → 样本分区分布 / 样本建模分
</commit_message>
<xml_diff>
--- a/report_100k.xlsx
+++ b/report_100k.xlsx
@@ -473,7 +473,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>partition_distribution</t>
+          <t>样本分区分布</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>modeling_score</t>
+          <t>样本建模分</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Sheet 2 variable filter summary table
Add 变量筛选 section at bottom of Sheet 2 with cumulative counts:
- 粗筛: PSI < 0.06, 缺失率 < 0.10, IV > 0.15, 相关性一致, 单调性
- 逐步回归: VIF < 3, VIF < 4, P-value < 0.01 (scorecard only)
- Each row shows remaining variable count after cumulative filtering

95 tests pass.
</commit_message>
<xml_diff>
--- a/report_100k.xlsx
+++ b/report_100k.xlsx
@@ -1069,13 +1069,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:S90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
@@ -1085,6 +1085,12 @@
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1160,6 +1166,36 @@
           <t>psi</t>
         </is>
       </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>_missing_max</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>_iv_num</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>_psi_num</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>_ks_train_num</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>_ks_oot_num</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>_monotonic</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -1213,6 +1249,24 @@
           <t>0.0007</t>
         </is>
       </c>
+      <c r="N3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="R3" s="3" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="S3" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -1266,6 +1320,24 @@
           <t>0.0006</t>
         </is>
       </c>
+      <c r="N4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="S4" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1319,6 +1391,24 @@
           <t>0.0007</t>
         </is>
       </c>
+      <c r="N5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="S5" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -1372,6 +1462,24 @@
           <t>0.0016</t>
         </is>
       </c>
+      <c r="N6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="S6" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -1425,6 +1533,24 @@
           <t>0.0005</t>
         </is>
       </c>
+      <c r="N7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="S7" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1478,6 +1604,24 @@
           <t>0.0003</t>
         </is>
       </c>
+      <c r="N8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="S8" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1531,6 +1675,24 @@
           <t>0.0002</t>
         </is>
       </c>
+      <c r="N9" s="3" t="n">
+        <v>0.0305</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="S9" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1584,6 +1746,24 @@
           <t>0.0008</t>
         </is>
       </c>
+      <c r="N10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="S10" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1637,6 +1817,24 @@
           <t>0.0001</t>
         </is>
       </c>
+      <c r="N11" s="3" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="S11" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -4105,6 +4303,135 @@
       </c>
       <c r="L82" s="4" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>变量筛选</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>筛选阶段</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>阈值</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>剩余变量数</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>粗筛</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>PSI</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>&lt;0.06</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>粗筛</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>缺失率</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>&lt;0.10</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>粗筛</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0.15</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>粗筛</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>与目标相关性</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>训练/验证前后一致</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>粗筛</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>业务解释</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>WOE单调性符合逻辑</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: sheet numbering, section numbering, filter count, WOE desc
1. 变量筛选: added 剩余变量数 column (all 0)
2. Sheet names: 1.模型设计 / 2.变量分析 / 3.模型表现
3. Section titles: 1.1/1.2/1.3, 2.1/2.2/2.3, 3.1/3.2/3.3/3.4, left-aligned
4. WOE tables: variable name + description from metadata

95 tests pass.
</commit_message>
<xml_diff>
--- a/report_100k.xlsx
+++ b/report_100k.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型设计" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变量分析" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型表现" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.模型设计" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.变量分析" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.模型表现" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>样本分区分布</t>
+          <t>1.1 样本分区分布</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>样本建模分</t>
+          <t>1.2 样本建模分</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>模型效果汇总</t>
+          <t>1.3 模型效果汇总</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>变量筛选</t>
+          <t>2.1 变量筛选</t>
         </is>
       </c>
     </row>
@@ -1110,6 +1110,11 @@
           <t>阈值</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>剩余变量数</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1127,6 +1132,9 @@
           <t>&lt;0.10</t>
         </is>
       </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1144,6 +1152,9 @@
           <t>&lt;0.30</t>
         </is>
       </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1161,6 +1172,9 @@
           <t>&gt;0.10</t>
         </is>
       </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1178,6 +1192,9 @@
           <t>训练/验证前后一致</t>
         </is>
       </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1195,6 +1212,9 @@
           <t>WOE单调性与目标符合逻辑</t>
         </is>
       </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1212,6 +1232,9 @@
           <t>&lt;0.3</t>
         </is>
       </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1229,6 +1252,9 @@
           <t>&lt;4</t>
         </is>
       </c>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1246,11 +1272,14 @@
           <t>&lt;0.01</t>
         </is>
       </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>变量总览</t>
+          <t>2.2 变量总览</t>
         </is>
       </c>
     </row>
@@ -4546,7 +4575,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>建模样本集效果</t>
+          <t>3.2 建模样本集效果</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4888,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>回溯效果</t>
+          <t>3.3 回溯效果</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: WOE data bars center at 0 (start_value=0), negative← positive→
- WOE column: start_type='num', start_value=0 → bars centered at zero
- bad_rate/lift/cum_lift: keep min/max proportional bars
- v1.0.2
</commit_message>
<xml_diff>
--- a/report_100k.xlsx
+++ b/report_100k.xlsx
@@ -4316,7 +4316,7 @@
   <conditionalFormatting sqref="I27:I33">
     <cfRule type="dataBar" priority="2">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4343,7 +4343,7 @@
   <conditionalFormatting sqref="I37:I41">
     <cfRule type="dataBar" priority="5">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4370,7 +4370,7 @@
   <conditionalFormatting sqref="I45:I48">
     <cfRule type="dataBar" priority="8">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4397,7 +4397,7 @@
   <conditionalFormatting sqref="I52:I54">
     <cfRule type="dataBar" priority="11">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4424,7 +4424,7 @@
   <conditionalFormatting sqref="I58:I62">
     <cfRule type="dataBar" priority="14">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4451,7 +4451,7 @@
   <conditionalFormatting sqref="I66:I72">
     <cfRule type="dataBar" priority="17">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4478,7 +4478,7 @@
   <conditionalFormatting sqref="I76:I80">
     <cfRule type="dataBar" priority="20">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4505,7 +4505,7 @@
   <conditionalFormatting sqref="I84:I87">
     <cfRule type="dataBar" priority="23">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>
@@ -4532,7 +4532,7 @@
   <conditionalFormatting sqref="I91:I94">
     <cfRule type="dataBar" priority="26">
       <dataBar minLength="5" maxLength="100" showValue="1">
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
       </dataBar>

</xml_diff>